<commit_message>
Finish Descriptive analyisis and store graphs and improve cleaning script further
</commit_message>
<xml_diff>
--- a/datasets/cleaned_response_dataset.xlsx
+++ b/datasets/cleaned_response_dataset.xlsx
@@ -448,7 +448,7 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>normal_use_battery_life</t>
+          <t>normal_use_battery_life(hours)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -468,12 +468,12 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>storage_capacity</t>
+          <t>storage_capacity(GB)</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>expected_life_span</t>
+          <t>expected_life_span(years)</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
@@ -488,7 +488,7 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>weight(g)</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>ram_capacity</t>
+          <t>ram_capacity(GB)</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>~2 hours</t>
+          <t>~2 Hours</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -700,7 +700,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>~2 hours</t>
+          <t>~2 Hours</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -772,7 +772,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2 weeks</t>
+          <t>2 Weeks</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1186,14 +1186,14 @@
         <v>12</v>
       </c>
       <c r="H11" t="n">
-        <v>7000000</v>
+        <v>70000</v>
       </c>
       <c r="I11" t="n">
-        <v>7000000</v>
+        <v>70000</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K11" t="n">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1258,14 +1258,14 @@
         <v>12</v>
       </c>
       <c r="H12" t="n">
-        <v>119</v>
+        <v>119999</v>
       </c>
       <c r="I12" t="n">
-        <v>119</v>
+        <v>119999</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K12" t="n">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K13" t="n">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1564,12 +1564,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>recommendation from a friend</t>
+          <t>Recommendation From A Friend</t>
         </is>
       </c>
       <c r="O16" t="n">
@@ -1618,10 +1618,10 @@
         <v>5</v>
       </c>
       <c r="H17" t="n">
-        <v>100</v>
+        <v>100000</v>
       </c>
       <c r="I17" t="n">
-        <v>180</v>
+        <v>180000</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2356,12 +2356,12 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>recommendation from a friend</t>
+          <t>Recommendation From A Friend</t>
         </is>
       </c>
       <c r="O27" t="n">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2626,10 +2626,10 @@
         <v>5</v>
       </c>
       <c r="H31" t="n">
-        <v>350</v>
+        <v>350000</v>
       </c>
       <c r="I31" t="n">
-        <v>395</v>
+        <v>395000</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K32" t="n">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2788,12 +2788,12 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>recommendation from a friend</t>
+          <t>Recommendation From A Friend</t>
         </is>
       </c>
       <c r="O33" t="n">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Honor </t>
+          <t>Honor</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3766,7 +3766,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K47" t="n">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3857,7 +3857,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K48" t="n">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>MSI (laotop)</t>
+          <t>Msi (Laotop)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4285,7 +4285,7 @@
         <v>200000</v>
       </c>
       <c r="I54" t="n">
-        <v>100000</v>
+        <v>165000</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4930,10 +4930,10 @@
         <v>12</v>
       </c>
       <c r="H63" t="n">
-        <v>350</v>
+        <v>350000</v>
       </c>
       <c r="I63" t="n">
-        <v>300</v>
+        <v>300000</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -5081,7 +5081,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K65" t="n">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -5452,7 +5452,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5494,7 +5494,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5524,7 +5524,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -5566,12 +5566,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Its speed what i wanted</t>
+          <t>Its Speed What I Wanted</t>
         </is>
       </c>
       <c r="G72" t="n">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -5668,12 +5668,12 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>recommendation from a friend</t>
+          <t>Recommendation From A Friend</t>
         </is>
       </c>
       <c r="O73" t="n">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K76" t="n">
@@ -5884,12 +5884,12 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>recommendation from a friend</t>
+          <t>Recommendation From A Friend</t>
         </is>
       </c>
       <c r="O76" t="n">
@@ -5916,7 +5916,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5926,7 +5926,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vivo </t>
+          <t>Vivo</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -5956,7 +5956,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -6017,7 +6017,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K78" t="n">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6089,7 +6089,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K79" t="n">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6244,7 +6244,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6316,7 +6316,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K87" t="n">
@@ -6676,7 +6676,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -6820,7 +6820,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -6892,7 +6892,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -6953,7 +6953,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K91" t="n">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -7068,7 +7068,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -7180,7 +7180,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -7252,7 +7252,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -7324,7 +7324,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -7396,7 +7396,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -7529,7 +7529,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K99" t="n">
@@ -7540,7 +7540,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -7594,7 +7594,7 @@
         <v>5</v>
       </c>
       <c r="H100" t="n">
-        <v>6000000</v>
+        <v>600000</v>
       </c>
       <c r="I100" t="n">
         <v>50000</v>
@@ -7612,7 +7612,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -7684,7 +7684,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -7756,7 +7756,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -7798,7 +7798,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -7810,10 +7810,10 @@
         <v>10</v>
       </c>
       <c r="H103" t="n">
-        <v>320</v>
+        <v>320000</v>
       </c>
       <c r="I103" t="n">
-        <v>320</v>
+        <v>320000</v>
       </c>
       <c r="J103" t="inlineStr">
         <is>
@@ -7828,7 +7828,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -7900,7 +7900,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -7972,7 +7972,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -8044,7 +8044,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -8116,7 +8116,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -8201,7 +8201,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>for Academic works</t>
+          <t>For Academic Works</t>
         </is>
       </c>
       <c r="Q108" t="n">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -8332,7 +8332,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -8386,10 +8386,10 @@
         <v>5</v>
       </c>
       <c r="H111" t="n">
-        <v>400</v>
+        <v>400000</v>
       </c>
       <c r="I111" t="n">
-        <v>380</v>
+        <v>380000</v>
       </c>
       <c r="J111" t="inlineStr">
         <is>
@@ -8404,7 +8404,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -8436,7 +8436,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -8476,7 +8476,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -8530,14 +8530,14 @@
         <v>3</v>
       </c>
       <c r="H113" t="n">
-        <v>220</v>
+        <v>220000</v>
       </c>
       <c r="I113" t="n">
-        <v>250</v>
+        <v>250000</v>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K113" t="n">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -8681,7 +8681,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K115" t="n">
@@ -8692,7 +8692,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -8764,7 +8764,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -8796,7 +8796,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -8836,7 +8836,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -8897,7 +8897,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K118" t="n">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -8980,7 +8980,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -9052,7 +9052,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -9084,7 +9084,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -9106,10 +9106,10 @@
         <v>12</v>
       </c>
       <c r="H121" t="n">
-        <v>5000000</v>
+        <v>50000</v>
       </c>
       <c r="I121" t="n">
-        <v>5000000</v>
+        <v>50000</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
@@ -9124,7 +9124,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -9196,7 +9196,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -9268,7 +9268,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -9340,7 +9340,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -9372,7 +9372,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -9397,7 +9397,7 @@
         <v>150000</v>
       </c>
       <c r="I125" t="n">
-        <v>150</v>
+        <v>150000</v>
       </c>
       <c r="J125" t="inlineStr">
         <is>
@@ -9412,7 +9412,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -9444,7 +9444,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -9628,7 +9628,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -9700,7 +9700,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -9732,7 +9732,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -9772,7 +9772,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -9804,7 +9804,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -9876,7 +9876,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -9905,7 +9905,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K132" t="n">
@@ -9916,7 +9916,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -9948,7 +9948,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -9988,7 +9988,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -10060,7 +10060,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -10132,7 +10132,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -10164,7 +10164,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -10204,7 +10204,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N136" t="inlineStr">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -10276,7 +10276,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>It has a privacy protector</t>
+          <t>It Has A Privacy Protector</t>
         </is>
       </c>
       <c r="G138" t="n">
@@ -10337,7 +10337,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K138" t="n">
@@ -10348,7 +10348,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
@@ -10405,7 +10405,7 @@
         <v>200000</v>
       </c>
       <c r="I139" t="n">
-        <v>215</v>
+        <v>215000</v>
       </c>
       <c r="J139" t="inlineStr">
         <is>
@@ -10420,7 +10420,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
@@ -10492,7 +10492,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -10524,7 +10524,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -10549,7 +10549,7 @@
         <v>20000</v>
       </c>
       <c r="I141" t="n">
-        <v>2000000</v>
+        <v>20000</v>
       </c>
       <c r="J141" t="inlineStr">
         <is>
@@ -10564,7 +10564,7 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>I didn't research before purchase</t>
+          <t>I Didn'T Research Before Purchase</t>
         </is>
       </c>
       <c r="N141" t="inlineStr">
@@ -10636,7 +10636,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N142" t="inlineStr">
@@ -10708,7 +10708,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
@@ -10780,7 +10780,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -10852,7 +10852,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -10981,7 +10981,7 @@
         <v>180000</v>
       </c>
       <c r="I147" t="n">
-        <v>163</v>
+        <v>163000</v>
       </c>
       <c r="J147" t="inlineStr">
         <is>
@@ -10996,7 +10996,7 @@
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -11028,7 +11028,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -11057,7 +11057,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K148" t="n">
@@ -11068,7 +11068,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>MSI</t>
+          <t>Msi</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -11194,10 +11194,10 @@
         <v>3</v>
       </c>
       <c r="H150" t="n">
-        <v>250</v>
+        <v>250000</v>
       </c>
       <c r="I150" t="n">
-        <v>234</v>
+        <v>234000</v>
       </c>
       <c r="J150" t="inlineStr">
         <is>
@@ -11212,7 +11212,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -11284,7 +11284,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>only few hours</t>
+          <t>Only Few Hours</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -11388,7 +11388,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Faculty Of Humanities and Social Sciences</t>
+          <t>Faculty Of Humanities And Social Sciences</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -11410,14 +11410,14 @@
         <v>10</v>
       </c>
       <c r="H153" t="n">
-        <v>300</v>
+        <v>300000</v>
       </c>
       <c r="I153" t="n">
-        <v>245</v>
+        <v>245000</v>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K153" t="n">
@@ -11428,7 +11428,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -11500,7 +11500,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -11572,7 +11572,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samsung </t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -11644,7 +11644,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -11716,7 +11716,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -11777,7 +11777,7 @@
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>Card Full Payment (Credit or Debit)</t>
+          <t>Card Full Payment (Credit Or Debit)</t>
         </is>
       </c>
       <c r="K158" t="n">
@@ -11788,7 +11788,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>few weeks</t>
+          <t>Few Weeks</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -11860,7 +11860,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>few months</t>
+          <t>Few Months</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>only few days</t>
+          <t>Only Few Days</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">

</xml_diff>